<commit_message>
l'ajout des methées de la génération des noms de fichiers et modification de la méthode calcul total factures prestataireÃ
</commit_message>
<xml_diff>
--- a/FinPay3/rapport_2026-02.xlsx
+++ b/FinPay3/rapport_2026-02.xlsx
@@ -6,36 +6,27 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" r:id="rId3" sheetId="1"/>
+    <sheet name="Rapport 2026-02" r:id="rId3" sheetId="1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>nom</t>
+    <t>Prestataire</t>
   </si>
   <si>
-    <t>Nombre_Factures</t>
+    <t>Nombre Factures</t>
   </si>
   <si>
-    <t>Total_Généré</t>
+    <t>Total Généré</t>
   </si>
   <si>
-    <t>Total_Commissions</t>
+    <t>Total Commissions</t>
   </si>
   <si>
-    <t>Prestataire Orange</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>300.00</t>
-  </si>
-  <si>
-    <t>6.0000</t>
+    <t>Tech Solutions</t>
   </si>
 </sst>
 </file>
@@ -101,14 +92,14 @@
       <c r="A2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>5</v>
+      <c r="B2" t="n" s="0">
+        <v>1.0</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>6</v>
+      <c r="C2" t="n" s="0">
+        <v>3.456789E7</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>7</v>
+      <c r="D2" t="n" s="0">
+        <v>691357.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>